<commit_message>
Update the MIM rows of Persona KPI Metrics Coverage for MIM V3
Each existing MIM KPI marked Pass / Partial / Fail against MIM V3, with the
reason in Explanation; the 23 KPIs MIM V3 achieves that the list lacked
added after the MIM rows. Edited in the sheet XML so the in-cell evidence
pictures and the other sheets are untouched.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UQEseLGdhSbfUn9TQsQUqG
</commit_message>
<xml_diff>
--- a/Dashboard Testing and Verification Template.xlsx
+++ b/Dashboard Testing and Verification Template.xlsx
@@ -22,7 +22,7 @@
     <sheet name="Dashbaord Review Feedback" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Persona KPI  Metrics Coverage'!$A$1:$S$152</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Persona KPI  Metrics Coverage'!$A$1:$S$175</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'SRE KPI  Metrics Coverage'!$B$1:$AK$40</definedName>
   </definedNames>
   <calcPr calcId="191028" iterateDelta="1E-4"/>
@@ -12593,7 +12593,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F8E8311-F168-4ED2-854F-F6B1C5578AEA}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:T152"/>
+  <dimension ref="A1:T175"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="17.7265625" style="5" customWidth="1"/>
@@ -18709,13 +18709,19 @@
       <c r="N122" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="O122" s="14" t="s">
-        <v>301</v>
+      <c r="O122" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partial</t>
+        </is>
       </c>
       <c r="P122" s="14"/>
       <c r="Q122" s="14"/>
       <c r="R122" s="14"/>
-      <c r="S122" s="14"/>
+      <c r="S122" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): Active P1 tile counts every active P1; P2s are counted only once open longer than 8 h (P2 over 8 h tile). There is no single P1 + P2 count. (Overall Status was Pass for the earlier MIM dashboard.)</t>
+        </is>
+      </c>
     </row>
     <row r="123" spans="1:19" s="4" customFormat="1">
       <c r="A123" s="14" t="s">
@@ -18758,13 +18764,19 @@
       <c r="N123" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="O123" s="14" t="s">
-        <v>301</v>
+      <c r="O123" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
       </c>
       <c r="P123" s="14"/>
       <c r="Q123" s="14"/>
       <c r="R123" s="14"/>
-      <c r="S123" s="14"/>
+      <c r="S123" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): No MTTR figure. The P1 / P2 / P3 trend now plots the age so far of New / In Progress incidents against the targets, not resolution times. (Overall Status was Pass for the earlier MIM dashboard.)</t>
+        </is>
+      </c>
     </row>
     <row r="124" spans="1:19" s="4" customFormat="1">
       <c r="A124" s="14" t="s">
@@ -18807,13 +18819,19 @@
       <c r="N124" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="O124" s="14" t="s">
-        <v>301</v>
+      <c r="O124" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
       </c>
       <c r="P124" s="14"/>
       <c r="Q124" s="14"/>
       <c r="R124" s="14"/>
-      <c r="S124" s="14"/>
+      <c r="S124" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): Not in MIM V3. (Overall Status was Pass for the earlier MIM dashboard.)</t>
+        </is>
+      </c>
     </row>
     <row r="125" spans="1:19" s="4" customFormat="1">
       <c r="A125" s="14" t="s">
@@ -18856,13 +18874,19 @@
       <c r="N125" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="O125" s="14" t="s">
-        <v>301</v>
+      <c r="O125" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
       </c>
       <c r="P125" s="14"/>
       <c r="Q125" s="14"/>
       <c r="R125" s="14"/>
-      <c r="S125" s="14"/>
+      <c r="S125" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): No total count of active incidents: the Active P1 / P2 / P3 donut was replaced by the Active P1, P2 over 8 h and P3 over 24 h tiles (25 Oct). (Overall Status was Pass for the earlier MIM dashboard.)</t>
+        </is>
+      </c>
     </row>
     <row r="126" spans="1:19" s="4" customFormat="1">
       <c r="A126" s="14" t="s">
@@ -18905,13 +18929,19 @@
       <c r="N126" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="O126" s="14" t="s">
-        <v>301</v>
+      <c r="O126" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partial</t>
+        </is>
       </c>
       <c r="P126" s="14"/>
       <c r="Q126" s="14"/>
       <c r="R126" s="14"/>
-      <c r="S126" s="14"/>
+      <c r="S126" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): No count. Breach is shown per incident in the Active Incidents SLA column (Breached = task_has_breached on its servicenow-task-sla records); only ~3 % of incidents have an SLA record in Elastic (Round 16). P2 over 8 h counts P2s past the target by age. (Overall Status was Pass for the earlier MIM dashboard.)</t>
+        </is>
+      </c>
     </row>
     <row r="127" spans="1:19" s="4" customFormat="1">
       <c r="A127" s="14" t="s">
@@ -18954,13 +18984,19 @@
       <c r="N127" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="O127" s="14" t="s">
-        <v>301</v>
+      <c r="O127" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partial</t>
+        </is>
       </c>
       <c r="P127" s="14"/>
       <c r="Q127" s="14"/>
       <c r="R127" s="14"/>
-      <c r="S127" s="14"/>
+      <c r="S127" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): No count. Shown per incident in the Active Incidents SLA column as "Breaching" (75 % of the SLA used or due within 30 min; 75 %, not 80 %). (Overall Status was Pass for the earlier MIM dashboard.)</t>
+        </is>
+      </c>
     </row>
     <row r="128" spans="1:19" s="4" customFormat="1">
       <c r="A128" s="14" t="s">
@@ -19003,13 +19039,19 @@
       <c r="N128" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="O128" s="14" t="s">
-        <v>301</v>
+      <c r="O128" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partial</t>
+        </is>
       </c>
       <c r="P128" s="14"/>
       <c r="Q128" s="14"/>
       <c r="R128" s="14"/>
-      <c r="S128" s="14"/>
+      <c r="S128" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): No count. Shown per incident in the Active Incidents SLA column as "Within SLA". (Overall Status was Pass for the earlier MIM dashboard.)</t>
+        </is>
+      </c>
     </row>
     <row r="129" spans="1:19" s="4" customFormat="1">
       <c r="A129" s="14" t="s">
@@ -19052,13 +19094,19 @@
       <c r="N129" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="O129" s="14" t="s">
-        <v>301</v>
+      <c r="O129" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
       </c>
       <c r="P129" s="14"/>
       <c r="Q129" s="14"/>
       <c r="R129" s="14"/>
-      <c r="S129" s="14"/>
+      <c r="S129" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): Not in MIM V3. (Overall Status was Pass for the earlier MIM dashboard.)</t>
+        </is>
+      </c>
     </row>
     <row r="130" spans="1:19" s="4" customFormat="1">
       <c r="A130" s="14" t="s">
@@ -19099,13 +19147,21 @@
       </c>
       <c r="M130" s="14"/>
       <c r="N130" s="14"/>
-      <c r="O130" s="14"/>
+      <c r="O130" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="P130" s="63" t="s">
         <v>688</v>
       </c>
       <c r="Q130" s="14"/>
       <c r="R130" s="14"/>
-      <c r="S130" s="14"/>
+      <c r="S130" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): Active Incidents (P1 · P2 over 8 h · P3 over 24 h): number, priority, CI, state, SLA (from servicenow-task-sla), assignment group, assignee, group manager and short description. P2 / P3 are listed only once past their 8 h / 24 h target.</t>
+        </is>
+      </c>
     </row>
     <row r="131" spans="1:19" s="4" customFormat="1">
       <c r="A131" s="14" t="s">
@@ -19148,13 +19204,21 @@
       <c r="N131" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="O131" s="14"/>
+      <c r="O131" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="P131" s="63" t="s">
         <v>692</v>
       </c>
       <c r="Q131" s="14"/>
       <c r="R131" s="14"/>
-      <c r="S131" s="14"/>
+      <c r="S131" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): Combined with the row above in Active Incidents (as noted); the CI support group per incident is in Escalate (section 2).</t>
+        </is>
+      </c>
     </row>
     <row r="132" spans="1:19" s="4" customFormat="1">
       <c r="A132" s="14" t="s">
@@ -19197,13 +19261,19 @@
       <c r="N132" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="O132" s="14" t="s">
-        <v>301</v>
+      <c r="O132" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partial</t>
+        </is>
       </c>
       <c r="P132" s="14"/>
       <c r="Q132" s="14"/>
       <c r="R132" s="14"/>
-      <c r="S132" s="14"/>
+      <c r="S132" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): P1 / P2 / P3 Time to Resolve vs Target: daily average (not median) for P1, P2 and P3 against 4 h / 8 h / 24 h lines, last 7 days. Since 27 Oct it covers New / In Progress incidents only (age so far), so it no longer shows resolution times. (Overall Status was Pass for the earlier MIM dashboard.)</t>
+        </is>
+      </c>
     </row>
     <row r="133" spans="1:19" s="4" customFormat="1">
       <c r="A133" s="14" t="s">
@@ -19246,13 +19316,19 @@
       <c r="N133" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="O133" s="14" t="s">
-        <v>301</v>
+      <c r="O133" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
       </c>
       <c r="P133" s="14"/>
       <c r="Q133" s="14"/>
       <c r="R133" s="14"/>
-      <c r="S133" s="14"/>
+      <c r="S133" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): Not in MIM V3. (Overall Status was Pass for the earlier MIM dashboard.)</t>
+        </is>
+      </c>
     </row>
     <row r="134" spans="1:19" s="4" customFormat="1">
       <c r="A134" s="14" t="s">
@@ -19295,13 +19371,19 @@
       <c r="N134" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="O134" s="14" t="s">
-        <v>301</v>
+      <c r="O134" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partial</t>
+        </is>
       </c>
       <c r="P134" s="14"/>
       <c r="Q134" s="14"/>
       <c r="R134" s="14"/>
-      <c r="S134" s="14"/>
+      <c r="S134" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): No per-CI counts. Active Incidents lists each incident with its CI; Escalate shows the picked CI's incidents and support group. (Overall Status was Pass for the earlier MIM dashboard.)</t>
+        </is>
+      </c>
     </row>
     <row r="135" spans="1:19" s="4" customFormat="1">
       <c r="A135" s="14" t="s">
@@ -19344,13 +19426,19 @@
       <c r="N135" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="O135" s="14" t="s">
-        <v>301</v>
+      <c r="O135" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
       </c>
       <c r="P135" s="14"/>
       <c r="Q135" s="14"/>
       <c r="R135" s="14"/>
-      <c r="S135" s="14"/>
+      <c r="S135" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): Not in MIM V3. (Overall Status was Pass for the earlier MIM dashboard.)</t>
+        </is>
+      </c>
     </row>
     <row r="136" spans="1:19" s="4" customFormat="1">
       <c r="A136" s="14" t="s">
@@ -19393,13 +19481,19 @@
       <c r="N136" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="O136" s="14" t="s">
-        <v>301</v>
+      <c r="O136" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
       </c>
       <c r="P136" s="14"/>
       <c r="Q136" s="14"/>
       <c r="R136" s="14"/>
-      <c r="S136" s="14"/>
+      <c r="S136" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): Not in MIM V3 (contact_type is not used). (Overall Status was Pass for the earlier MIM dashboard.)</t>
+        </is>
+      </c>
     </row>
     <row r="137" spans="1:19" s="4" customFormat="1">
       <c r="A137" s="14" t="s">
@@ -19442,13 +19536,19 @@
       <c r="N137" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="O137" s="14" t="s">
-        <v>301</v>
+      <c r="O137" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
       </c>
       <c r="P137" s="14"/>
       <c r="Q137" s="14"/>
       <c r="R137" s="14"/>
-      <c r="S137" s="14"/>
+      <c r="S137" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): No breakdown by assignment group; the group is shown per incident in Active Incidents and Escalate. (Overall Status was Pass for the earlier MIM dashboard.)</t>
+        </is>
+      </c>
     </row>
     <row r="138" spans="1:19" s="4" customFormat="1">
       <c r="A138" s="14" t="s">
@@ -19491,13 +19591,19 @@
       <c r="N138" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="O138" s="14" t="s">
-        <v>301</v>
+      <c r="O138" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
       </c>
       <c r="P138" s="14"/>
       <c r="Q138" s="14"/>
       <c r="R138" s="14"/>
-      <c r="S138" s="14"/>
+      <c r="S138" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): Not in MIM V3. (Overall Status was Pass for the earlier MIM dashboard.)</t>
+        </is>
+      </c>
     </row>
     <row r="139" spans="1:19" customFormat="1">
       <c r="A139" s="14" t="s">
@@ -19540,681 +19646,2458 @@
       <c r="N139" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="O139" s="14" t="s">
-        <v>301</v>
+      <c r="O139" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
       </c>
       <c r="P139" s="14"/>
       <c r="Q139" s="14"/>
       <c r="R139" s="14"/>
-      <c r="S139" s="14"/>
-    </row>
-    <row r="140" spans="1:19" customFormat="1" hidden="1">
-      <c r="A140" s="14" t="s">
-        <v>723</v>
-      </c>
-      <c r="B140" s="14" t="s">
-        <v>490</v>
-      </c>
-      <c r="C140" s="14" t="s">
-        <v>545</v>
-      </c>
-      <c r="D140" s="14" t="s">
-        <v>516</v>
-      </c>
-      <c r="E140" s="64" t="s">
-        <v>315</v>
-      </c>
-      <c r="F140" s="14" t="s">
-        <v>316</v>
-      </c>
-      <c r="G140" s="14" t="s">
-        <v>392</v>
-      </c>
-      <c r="H140" s="14" t="s">
-        <v>318</v>
-      </c>
-      <c r="I140" s="14" t="s">
-        <v>546</v>
-      </c>
-      <c r="J140" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="K140" s="14" t="s">
-        <v>315</v>
-      </c>
-      <c r="L140" s="14" t="e" vm="112">
-        <v>#VALUE!</v>
-      </c>
+      <c r="S139" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): Not in MIM V3. (Overall Status was Pass for the earlier MIM dashboard.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" spans="1:19">
+      <c r="A140" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B140" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview</t>
+        </is>
+      </c>
+      <c r="C140" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Active P1 incidents</t>
+        </is>
+      </c>
+      <c r="D140" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Every active P1 incident, whatever its age</t>
+        </is>
+      </c>
+      <c r="E140" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">count</t>
+        </is>
+      </c>
+      <c r="F140" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">logs</t>
+        </is>
+      </c>
+      <c r="G140" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">servicenow-incidents</t>
+        </is>
+      </c>
+      <c r="H140" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Active P1 (Metric)</t>
+        </is>
+      </c>
+      <c r="I140" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Each incident judged on its latest record; active = state not On Hold, Resolved, Closed, Canceled or Cancelled. Last 7 days (fixed).</t>
+        </is>
+      </c>
+      <c r="J140" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="K140" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">count</t>
+        </is>
+      </c>
+      <c r="L140" s="14"/>
       <c r="M140" s="14"/>
-      <c r="N140" s="14" t="s">
-        <v>408</v>
-      </c>
-      <c r="O140" s="14" t="s">
-        <v>301</v>
-      </c>
-      <c r="P140" s="14" t="s">
-        <v>547</v>
-      </c>
+      <c r="N140" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O140" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P140" s="14"/>
       <c r="Q140" s="14"/>
       <c r="R140" s="14"/>
-      <c r="S140" s="14"/>
-    </row>
-    <row r="141" spans="1:19" hidden="1">
-      <c r="A141" s="14" t="s">
-        <v>723</v>
-      </c>
-      <c r="B141" s="14" t="s">
-        <v>490</v>
-      </c>
-      <c r="C141" s="14" t="s">
-        <v>548</v>
-      </c>
-      <c r="D141" s="14" t="s">
-        <v>549</v>
-      </c>
-      <c r="E141" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="F141" s="14" t="s">
-        <v>297</v>
-      </c>
-      <c r="G141" s="14" t="s">
-        <v>298</v>
-      </c>
-      <c r="H141" s="14" t="s">
-        <v>304</v>
-      </c>
-      <c r="I141" s="14" t="s">
-        <v>550</v>
-      </c>
-      <c r="J141" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="K141" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="L141" s="14" t="e" vm="113">
-        <v>#VALUE!</v>
-      </c>
+      <c r="S140" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 1); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" spans="1:19">
+      <c r="A141" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B141" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview</t>
+        </is>
+      </c>
+      <c r="C141" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2 incidents over 8 h target</t>
+        </is>
+      </c>
+      <c r="D141" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Active P2 incidents open longer than the 8 h target</t>
+        </is>
+      </c>
+      <c r="E141" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">count</t>
+        </is>
+      </c>
+      <c r="F141" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">logs</t>
+        </is>
+      </c>
+      <c r="G141" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">servicenow-incidents</t>
+        </is>
+      </c>
+      <c r="H141" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2 over 8 h (Metric)</t>
+        </is>
+      </c>
+      <c r="I141" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Age = now - opened_at &gt; 8 h; same active rule as Active P1.</t>
+        </is>
+      </c>
+      <c r="J141" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="K141" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">count</t>
+        </is>
+      </c>
+      <c r="L141" s="14"/>
       <c r="M141" s="14"/>
-      <c r="N141" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="O141" s="14" t="s">
-        <v>408</v>
-      </c>
-      <c r="P141" s="62" t="s">
-        <v>724</v>
-      </c>
+      <c r="N141" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O141" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P141" s="14"/>
       <c r="Q141" s="14"/>
       <c r="R141" s="14"/>
-      <c r="S141" s="14"/>
-    </row>
-    <row r="142" spans="1:19" hidden="1">
-      <c r="A142" s="14" t="s">
-        <v>723</v>
-      </c>
-      <c r="B142" s="14" t="s">
-        <v>490</v>
-      </c>
-      <c r="C142" s="14" t="s">
-        <v>551</v>
-      </c>
-      <c r="D142" s="14" t="s">
-        <v>552</v>
-      </c>
-      <c r="E142" s="14" t="s">
-        <v>553</v>
-      </c>
-      <c r="F142" s="14" t="s">
-        <v>297</v>
-      </c>
-      <c r="G142" s="14" t="s">
-        <v>554</v>
-      </c>
-      <c r="H142" s="14" t="s">
-        <v>318</v>
-      </c>
-      <c r="I142" s="14" t="s">
-        <v>555</v>
-      </c>
-      <c r="J142" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="K142" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="L142" s="14" t="e" vm="114">
-        <v>#VALUE!</v>
-      </c>
+      <c r="S141" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 1); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" spans="1:19">
+      <c r="A142" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B142" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview</t>
+        </is>
+      </c>
+      <c r="C142" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3 incidents over 24 h target</t>
+        </is>
+      </c>
+      <c r="D142" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Active P3 incidents open longer than the 24 h target</t>
+        </is>
+      </c>
+      <c r="E142" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">count</t>
+        </is>
+      </c>
+      <c r="F142" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">logs</t>
+        </is>
+      </c>
+      <c r="G142" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">servicenow-incidents</t>
+        </is>
+      </c>
+      <c r="H142" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3 over 24 h (Metric)</t>
+        </is>
+      </c>
+      <c r="I142" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Age = now - opened_at &gt; 24 h; same active rule as Active P1.</t>
+        </is>
+      </c>
+      <c r="J142" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="K142" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">count</t>
+        </is>
+      </c>
+      <c r="L142" s="14"/>
       <c r="M142" s="14"/>
-      <c r="N142" s="14" t="s">
-        <v>408</v>
-      </c>
-      <c r="O142" s="14" t="s">
-        <v>408</v>
-      </c>
-      <c r="P142" s="62" t="s">
-        <v>725</v>
-      </c>
+      <c r="N142" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O142" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P142" s="14"/>
       <c r="Q142" s="14"/>
       <c r="R142" s="14"/>
-      <c r="S142" s="14"/>
-    </row>
-    <row r="143" spans="1:19" hidden="1">
-      <c r="A143" s="14" t="s">
-        <v>723</v>
-      </c>
-      <c r="B143" s="14" t="s">
-        <v>490</v>
-      </c>
-      <c r="C143" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="D143" s="14" t="s">
-        <v>726</v>
-      </c>
-      <c r="E143" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="F143" s="14" t="s">
-        <v>316</v>
-      </c>
-      <c r="G143" s="14" t="s">
-        <v>392</v>
-      </c>
-      <c r="H143" s="14" t="s">
-        <v>304</v>
-      </c>
-      <c r="I143" s="14" t="s">
-        <v>727</v>
-      </c>
-      <c r="J143" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="K143" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="L143" s="14" t="e" vm="115">
-        <v>#VALUE!</v>
-      </c>
+      <c r="S142" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 1); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" spans="1:19">
+      <c r="A143" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B143" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview</t>
+        </is>
+      </c>
+      <c r="C143" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open alerts with no incident</t>
+        </is>
+      </c>
+      <c r="D143" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Netcool alerts still open on a CI that has no open incident</t>
+        </is>
+      </c>
+      <c r="E143" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="F143" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">logs</t>
+        </is>
+      </c>
+      <c r="G143" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">.ds-bridge-alerts-netcool-default-*, servicenow-incidents</t>
+        </is>
+      </c>
+      <c r="H143" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open Alerts with No Incident (Table)</t>
+        </is>
+      </c>
+      <c r="I143" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open = latest record is not a clear / resolution. Critical first. Last 24 h.</t>
+        </is>
+      </c>
+      <c r="J143" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CI, node, severity, alert, times fired, first / last seen</t>
+        </is>
+      </c>
+      <c r="K143" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="L143" s="14"/>
       <c r="M143" s="14"/>
-      <c r="N143" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="O143" s="14" t="s">
-        <v>66</v>
+      <c r="N143" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O143" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
       </c>
       <c r="P143" s="14"/>
       <c r="Q143" s="14"/>
       <c r="R143" s="14"/>
-      <c r="S143" s="14"/>
-    </row>
-    <row r="144" spans="1:19" hidden="1">
-      <c r="A144" s="14" t="s">
-        <v>723</v>
-      </c>
-      <c r="B144" s="14" t="s">
-        <v>490</v>
-      </c>
-      <c r="C144" s="14" t="s">
-        <v>557</v>
-      </c>
-      <c r="D144" s="14" t="s">
-        <v>558</v>
-      </c>
-      <c r="E144" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="F144" s="14" t="s">
-        <v>297</v>
-      </c>
-      <c r="G144" s="14" t="s">
-        <v>298</v>
-      </c>
-      <c r="H144" s="14" t="s">
-        <v>427</v>
-      </c>
-      <c r="I144" s="14" t="s">
-        <v>559</v>
-      </c>
-      <c r="J144" s="14" t="s">
-        <v>560</v>
-      </c>
-      <c r="K144" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="L144" s="14" t="e" vm="116">
-        <v>#VALUE!</v>
-      </c>
+      <c r="S143" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 1); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" spans="1:19">
+      <c r="A144" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B144" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detailed</t>
+        </is>
+      </c>
+      <c r="C144" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Who to escalate to</t>
+        </is>
+      </c>
+      <c r="D144" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Active incidents on the selected CI with the CI support group, assignment group, assignee and group manager</t>
+        </is>
+      </c>
+      <c r="E144" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="F144" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">logs, metrics</t>
+        </is>
+      </c>
+      <c r="G144" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">servicenow-incidents, metrics-system.cpu (CMDB enrichment)</t>
+        </is>
+      </c>
+      <c r="H144" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Escalate (Table)</t>
+        </is>
+      </c>
+      <c r="I144" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Follows the Incident / CI controls. Last 7 days.</t>
+        </is>
+      </c>
+      <c r="J144" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CI, incident, priority, class, environment, support group, assignment group, assignee, group manager (with emails)</t>
+        </is>
+      </c>
+      <c r="K144" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="L144" s="14"/>
       <c r="M144" s="14"/>
-      <c r="N144" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="O144" s="14" t="s">
-        <v>301</v>
-      </c>
-      <c r="P144" s="14" t="s">
-        <v>728</v>
-      </c>
+      <c r="N144" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O144" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P144" s="14"/>
       <c r="Q144" s="14"/>
       <c r="R144" s="14"/>
-      <c r="S144" s="14"/>
-    </row>
-    <row r="145" spans="1:19" hidden="1">
-      <c r="A145" s="14" t="s">
-        <v>723</v>
-      </c>
-      <c r="B145" s="14" t="s">
-        <v>490</v>
-      </c>
-      <c r="C145" s="14" t="s">
-        <v>729</v>
-      </c>
-      <c r="D145" s="14" t="s">
-        <v>562</v>
-      </c>
-      <c r="E145" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="F145" s="14" t="s">
-        <v>297</v>
-      </c>
-      <c r="G145" s="14" t="s">
-        <v>298</v>
-      </c>
-      <c r="H145" s="14" t="s">
-        <v>304</v>
-      </c>
-      <c r="I145" s="14" t="s">
-        <v>563</v>
-      </c>
-      <c r="J145" s="14" t="s">
-        <v>564</v>
-      </c>
-      <c r="K145" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="L145" s="14" t="e" vm="117">
-        <v>#VALUE!</v>
-      </c>
+      <c r="S144" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 2); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" spans="1:19">
+      <c r="A145" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B145" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detailed</t>
+        </is>
+      </c>
+      <c r="C145" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Changes on the CI</t>
+        </is>
+      </c>
+      <c r="D145" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Change requests with activity in the last 7 days on the selected CI and on CIs linked to it in the CMDB</t>
+        </is>
+      </c>
+      <c r="E145" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="F145" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">logs</t>
+        </is>
+      </c>
+      <c r="G145" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">servicenow-change-requests, cmdb-ci-relations</t>
+        </is>
+      </c>
+      <c r="H145" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Changes in the Last 7 Days on this CI (Table)</t>
+        </is>
+      </c>
+      <c r="I145" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Changes on linked CIs show only when their CMDB link was recorded in the same 7 days.</t>
+        </is>
+      </c>
+      <c r="J145" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">change, CI, type, category, state, outcome, planned start, end, group</t>
+        </is>
+      </c>
+      <c r="K145" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="L145" s="14"/>
       <c r="M145" s="14"/>
-      <c r="N145" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="O145" s="14" t="s">
-        <v>301</v>
-      </c>
-      <c r="P145" s="14" t="s">
-        <v>728</v>
-      </c>
+      <c r="N145" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O145" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P145" s="14"/>
       <c r="Q145" s="14"/>
       <c r="R145" s="14"/>
-      <c r="S145" s="14"/>
-    </row>
-    <row r="146" spans="1:19" hidden="1">
-      <c r="A146" s="14" t="s">
-        <v>723</v>
-      </c>
-      <c r="B146" s="14" t="s">
-        <v>490</v>
-      </c>
-      <c r="C146" s="14" t="s">
-        <v>566</v>
-      </c>
-      <c r="D146" s="14" t="s">
-        <v>567</v>
-      </c>
-      <c r="E146" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="F146" s="14" t="s">
-        <v>297</v>
-      </c>
-      <c r="G146" s="14" t="s">
-        <v>426</v>
-      </c>
-      <c r="H146" s="14" t="s">
-        <v>359</v>
-      </c>
-      <c r="I146" s="14" t="s">
-        <v>568</v>
-      </c>
-      <c r="J146" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="K146" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="L146" s="14" t="e" vm="118">
-        <v>#VALUE!</v>
-      </c>
+      <c r="S145" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 2); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" spans="1:19">
+      <c r="A146" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B146" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detailed</t>
+        </is>
+      </c>
+      <c r="C146" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alerts on the CI</t>
+        </is>
+      </c>
+      <c r="D146" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Netcool alerts on the selected CI, with when each started compared with the picked incident</t>
+        </is>
+      </c>
+      <c r="E146" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="F146" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">logs</t>
+        </is>
+      </c>
+      <c r="G146" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">.ds-bridge-alerts-netcool-default-*, servicenow-incidents</t>
+        </is>
+      </c>
+      <c r="H146" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alerts on this CI (Table)</t>
+        </is>
+      </c>
+      <c r="I146" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Likely trigger = first seen up to 2 h before the incident opened. Alerts: last 7 days.</t>
+        </is>
+      </c>
+      <c r="J146" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">state, severity, alert, vs incident, first / last seen, times fired, acknowledged</t>
+        </is>
+      </c>
+      <c r="K146" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="L146" s="14"/>
       <c r="M146" s="14"/>
-      <c r="N146" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="O146" s="14" t="s">
-        <v>408</v>
-      </c>
-      <c r="P146" s="14" t="s">
-        <v>569</v>
-      </c>
+      <c r="N146" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O146" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P146" s="14"/>
       <c r="Q146" s="14"/>
       <c r="R146" s="14"/>
-      <c r="S146" s="14"/>
-    </row>
-    <row r="147" spans="1:19" hidden="1">
-      <c r="A147" s="14" t="s">
-        <v>723</v>
-      </c>
-      <c r="B147" s="14" t="s">
-        <v>490</v>
-      </c>
-      <c r="C147" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="D147" s="14" t="s">
-        <v>570</v>
-      </c>
-      <c r="E147" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="F147" s="14" t="s">
-        <v>316</v>
-      </c>
-      <c r="G147" s="14" t="s">
-        <v>316</v>
-      </c>
-      <c r="H147" s="14" t="s">
-        <v>427</v>
-      </c>
-      <c r="I147" s="14" t="s">
-        <v>571</v>
-      </c>
-      <c r="J147" s="14"/>
-      <c r="K147" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="L147" s="14" t="e" vm="119">
-        <v>#VALUE!</v>
-      </c>
+      <c r="S146" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 2); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" spans="1:19">
+      <c r="A147" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B147" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detailed</t>
+        </is>
+      </c>
+      <c r="C147" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Blast radius</t>
+        </is>
+      </c>
+      <c r="D147" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Number of applications that depend directly on the selected CI</t>
+        </is>
+      </c>
+      <c r="E147" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">count</t>
+        </is>
+      </c>
+      <c r="F147" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CMDB</t>
+        </is>
+      </c>
+      <c r="G147" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cmdb-ci-relations</t>
+        </is>
+      </c>
+      <c r="H147" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Blast radius (Metric)</t>
+        </is>
+      </c>
+      <c r="I147" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Amber from 1, red from 5. Production only; retired applications left out.</t>
+        </is>
+      </c>
+      <c r="J147" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="K147" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">count</t>
+        </is>
+      </c>
+      <c r="L147" s="14"/>
       <c r="M147" s="14"/>
-      <c r="N147" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="O147" s="14" t="s">
-        <v>408</v>
-      </c>
-      <c r="P147" s="14" t="s">
-        <v>572</v>
-      </c>
+      <c r="N147" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O147" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P147" s="14"/>
       <c r="Q147" s="14"/>
       <c r="R147" s="14"/>
-      <c r="S147" s="14"/>
-    </row>
-    <row r="148" spans="1:19" hidden="1">
-      <c r="A148" s="14" t="s">
-        <v>723</v>
-      </c>
-      <c r="B148" s="14" t="s">
-        <v>490</v>
-      </c>
-      <c r="C148" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="D148" s="59" t="s">
-        <v>573</v>
-      </c>
-      <c r="E148" s="14" t="s">
-        <v>315</v>
-      </c>
-      <c r="F148" s="14" t="s">
-        <v>334</v>
-      </c>
-      <c r="G148" s="14" t="s">
-        <v>574</v>
-      </c>
-      <c r="H148" s="14" t="s">
-        <v>304</v>
-      </c>
-      <c r="I148" s="14" t="s">
-        <v>575</v>
-      </c>
-      <c r="J148" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="K148" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="L148" s="14" t="e" vm="120">
-        <v>#VALUE!</v>
-      </c>
+      <c r="S147" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 2); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" spans="1:19">
+      <c r="A148" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B148" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detailed</t>
+        </is>
+      </c>
+      <c r="C148" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Applications related to the CI</t>
+        </is>
+      </c>
+      <c r="D148" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Business applications, application services and instances related to the selected CI in the CMDB</t>
+        </is>
+      </c>
+      <c r="E148" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="F148" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CMDB</t>
+        </is>
+      </c>
+      <c r="G148" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cmdb-ci-relations</t>
+        </is>
+      </c>
+      <c r="H148" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Applications related to this CI (Table)</t>
+        </is>
+      </c>
+      <c r="I148" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Both directions; business applications first; retired marked.</t>
+        </is>
+      </c>
+      <c r="J148" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">application, kind, how related</t>
+        </is>
+      </c>
+      <c r="K148" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="L148" s="14"/>
       <c r="M148" s="14"/>
-      <c r="N148" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="O148" s="14" t="s">
-        <v>408</v>
-      </c>
-      <c r="P148" s="14" t="s">
-        <v>730</v>
-      </c>
+      <c r="N148" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O148" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P148" s="14"/>
       <c r="Q148" s="14"/>
       <c r="R148" s="14"/>
-      <c r="S148" s="14"/>
-    </row>
-    <row r="149" spans="1:19" hidden="1">
-      <c r="A149" s="14" t="s">
-        <v>723</v>
-      </c>
-      <c r="B149" s="14" t="s">
-        <v>490</v>
-      </c>
-      <c r="C149" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="D149" s="14" t="s">
-        <v>577</v>
-      </c>
-      <c r="E149" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="F149" s="14" t="s">
-        <v>297</v>
-      </c>
-      <c r="G149" s="59" t="s">
-        <v>298</v>
-      </c>
-      <c r="H149" s="14" t="s">
-        <v>427</v>
-      </c>
-      <c r="I149" s="14" t="s">
-        <v>578</v>
-      </c>
-      <c r="J149" s="14" t="s">
-        <v>564</v>
-      </c>
-      <c r="K149" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="L149" s="14" t="e" vm="121">
-        <v>#VALUE!</v>
-      </c>
+      <c r="S148" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 2); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" spans="1:19">
+      <c r="A149" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B149" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detailed</t>
+        </is>
+      </c>
+      <c r="C149" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Related CIs (middleware, database, server, other)</t>
+        </is>
+      </c>
+      <c r="D149" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Every CI related to the selected CI in the CMDB, by class</t>
+        </is>
+      </c>
+      <c r="E149" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="F149" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CMDB</t>
+        </is>
+      </c>
+      <c r="G149" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cmdb-ci-relations</t>
+        </is>
+      </c>
+      <c r="H149" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Middleware View, Database View, Server View, Other related CIs (Tables)</t>
+        </is>
+      </c>
+      <c r="I149" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Both directions, with the ServiceNow relationship; retired CIs listed last.</t>
+        </is>
+      </c>
+      <c r="J149" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">related CI, type, relationship, environment</t>
+        </is>
+      </c>
+      <c r="K149" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="L149" s="14"/>
       <c r="M149" s="14"/>
-      <c r="N149" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="O149" s="14" t="s">
-        <v>408</v>
-      </c>
-      <c r="P149" s="65" t="s">
-        <v>731</v>
-      </c>
+      <c r="N149" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O149" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P149" s="14"/>
       <c r="Q149" s="14"/>
       <c r="R149" s="14"/>
-      <c r="S149" s="14"/>
-    </row>
-    <row r="150" spans="1:19" hidden="1">
-      <c r="A150" s="14" t="s">
-        <v>723</v>
-      </c>
-      <c r="B150" s="14" t="s">
-        <v>490</v>
-      </c>
-      <c r="C150" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="D150" s="14" t="s">
-        <v>580</v>
-      </c>
-      <c r="E150" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="F150" s="14" t="s">
-        <v>297</v>
-      </c>
-      <c r="G150" s="59" t="s">
-        <v>298</v>
-      </c>
-      <c r="H150" s="14" t="s">
-        <v>304</v>
-      </c>
-      <c r="I150" s="14" t="s">
-        <v>581</v>
-      </c>
-      <c r="J150" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="K150" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="L150" s="14" t="e" vm="122">
-        <v>#VALUE!</v>
-      </c>
+      <c r="S149" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 2); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" spans="1:19">
+      <c r="A150" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B150" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detailed</t>
+        </is>
+      </c>
+      <c r="C150" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Application health (traffic light)</t>
+        </is>
+      </c>
+      <c r="D150" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Health of the production business applications related to the selected CI (all when none): Failing = a service with 10 % or more failed transactions, Degraded = 1 % or more, otherwise Healthy</t>
+        </is>
+      </c>
+      <c r="E150" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="F150" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">APM, CMDB</t>
+        </is>
+      </c>
+      <c r="G150" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metrics-apm.service_transaction.1m, metrics-apm.internal, cmdb-ci-relations, cmdb_with_apm_flag</t>
+        </is>
+      </c>
+      <c r="H150" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Application Health (Table)</t>
+        </is>
+      </c>
+      <c r="I150" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Last hour. Enrolled applications with no telemetry yet are listed last ("Enrolled - no telemetry yet").</t>
+        </is>
+      </c>
+      <c r="J150" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">application, health, servers, failing, degraded, services, worst service, app error rate, transactions, APM number, support group</t>
+        </is>
+      </c>
+      <c r="K150" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="L150" s="14"/>
       <c r="M150" s="14"/>
-      <c r="N150" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="O150" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="P150" s="61" t="s">
-        <v>582</v>
-      </c>
+      <c r="N150" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O150" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P150" s="14"/>
       <c r="Q150" s="14"/>
       <c r="R150" s="14"/>
-      <c r="S150" s="14"/>
-    </row>
-    <row r="151" spans="1:19" hidden="1">
-      <c r="A151" s="14" t="s">
-        <v>723</v>
-      </c>
-      <c r="B151" s="14" t="s">
-        <v>490</v>
-      </c>
-      <c r="C151" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="D151" s="14" t="s">
-        <v>583</v>
-      </c>
-      <c r="E151" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="F151" s="14" t="s">
-        <v>297</v>
-      </c>
-      <c r="G151" s="59" t="s">
-        <v>298</v>
-      </c>
-      <c r="H151" s="14" t="s">
-        <v>318</v>
-      </c>
-      <c r="I151" s="14" t="s">
-        <v>555</v>
-      </c>
-      <c r="J151" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="K151" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="L151" s="14" t="e" vm="123">
-        <v>#VALUE!</v>
-      </c>
+      <c r="S150" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 3); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" spans="1:19">
+      <c r="A151" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B151" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detailed</t>
+        </is>
+      </c>
+      <c r="C151" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Telemetry onboarding worklist</t>
+        </is>
+      </c>
+      <c r="D151" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Business applications enrolled for Elastic telemetry onboarding (is_monitored) that send no APM data yet</t>
+        </is>
+      </c>
+      <c r="E151" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">count</t>
+        </is>
+      </c>
+      <c r="F151" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CMDB, APM</t>
+        </is>
+      </c>
+      <c r="G151" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cmdb_with_apm_flag, metrics-apm.service_transaction.1m</t>
+        </is>
+      </c>
+      <c r="H151" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Application Health with the Telemetry control on "Enrolled, no telemetry yet" (Table)</t>
+        </is>
+      </c>
+      <c r="I151" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Matched on the application number; retired applications left out.</t>
+        </is>
+      </c>
+      <c r="J151" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">application, APM number, support group</t>
+        </is>
+      </c>
+      <c r="K151" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="L151" s="14"/>
       <c r="M151" s="14"/>
-      <c r="N151" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="O151" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="P151" s="61" t="s">
-        <v>582</v>
-      </c>
+      <c r="N151" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O151" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P151" s="14"/>
       <c r="Q151" s="14"/>
       <c r="R151" s="14"/>
-      <c r="S151" s="14"/>
-    </row>
-    <row r="152" spans="1:19" hidden="1">
-      <c r="A152" s="6" t="s">
+      <c r="S151" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 3); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" spans="1:19">
+      <c r="A152" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B152" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detailed</t>
+        </is>
+      </c>
+      <c r="C152" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Services of the application</t>
+        </is>
+      </c>
+      <c r="D152" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Services of the application picked in the Application control, worst first</t>
+        </is>
+      </c>
+      <c r="E152" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="F152" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">APM</t>
+        </is>
+      </c>
+      <c r="G152" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metrics-apm.service_transaction.1m, metrics-apm.internal</t>
+        </is>
+      </c>
+      <c r="H152" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Services of the Application (Table)</t>
+        </is>
+      </c>
+      <c r="I152" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Last hour; Low traffic = under 20 transactions, not rated.</t>
+        </is>
+      </c>
+      <c r="J152" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">service, application, servers, health, error rate, latency, per minute, transactions</t>
+        </is>
+      </c>
+      <c r="K152" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="L152" s="14"/>
+      <c r="M152" s="14"/>
+      <c r="N152" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O152" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P152" s="14"/>
+      <c r="Q152" s="14"/>
+      <c r="R152" s="14"/>
+      <c r="S152" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 3); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" spans="1:19">
+      <c r="A153" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B153" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detailed</t>
+        </is>
+      </c>
+      <c r="C153" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Upstream dependencies</t>
+        </is>
+      </c>
+      <c r="D153" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What the services in scope call (databases, queues, services) and how many of those calls failed</t>
+        </is>
+      </c>
+      <c r="E153" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="F153" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">APM</t>
+        </is>
+      </c>
+      <c r="G153" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metrics-apm.service_destination.1m, metrics-apm.internal</t>
+        </is>
+      </c>
+      <c r="H153" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Upstream - what they depend on (Bar)</t>
+        </is>
+      </c>
+      <c r="I153" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scope: the Service control, or the services on the selected CI. Last hour; top 15, failing first.</t>
+        </is>
+      </c>
+      <c r="J153" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dependency, calls, failed %</t>
+        </is>
+      </c>
+      <c r="K153" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="L153" s="14"/>
+      <c r="M153" s="14"/>
+      <c r="N153" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O153" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P153" s="14"/>
+      <c r="Q153" s="14"/>
+      <c r="R153" s="14"/>
+      <c r="S153" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 3); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" spans="1:19">
+      <c r="A154" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B154" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detailed</t>
+        </is>
+      </c>
+      <c r="C154" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Service health</t>
+        </is>
+      </c>
+      <c r="D154" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Share of failed transactions of each service in scope</t>
+        </is>
+      </c>
+      <c r="E154" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">%</t>
+        </is>
+      </c>
+      <c r="F154" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">APM</t>
+        </is>
+      </c>
+      <c r="G154" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metrics-apm.service_transaction.1m, metrics-apm.internal</t>
+        </is>
+      </c>
+      <c r="H154" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Service health (Tiles)</t>
+        </is>
+      </c>
+      <c r="I154" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Green / amber / red at 1 % and 10 %. Last hour.</t>
+        </is>
+      </c>
+      <c r="J154" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">service, business application</t>
+        </is>
+      </c>
+      <c r="K154" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">%</t>
+        </is>
+      </c>
+      <c r="L154" s="14"/>
+      <c r="M154" s="14"/>
+      <c r="N154" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O154" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P154" s="14"/>
+      <c r="Q154" s="14"/>
+      <c r="R154" s="14"/>
+      <c r="S154" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 3); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" spans="1:19">
+      <c r="A155" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B155" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detailed</t>
+        </is>
+      </c>
+      <c r="C155" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Downstream impact</t>
+        </is>
+      </c>
+      <c r="D155" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Production services that call the services in scope, and how many of their calls failed</t>
+        </is>
+      </c>
+      <c r="E155" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="F155" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">APM</t>
+        </is>
+      </c>
+      <c r="G155" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">traces-apm, metrics-apm.service_destination.1m</t>
+        </is>
+      </c>
+      <c r="H155" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Downstream - who is impacted (Bar)</t>
+        </is>
+      </c>
+      <c r="I155" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Matched on the host names the services answer on. Last hour; top 15, failing first.</t>
+        </is>
+      </c>
+      <c r="J155" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">calling service, calls, failed %</t>
+        </is>
+      </c>
+      <c r="K155" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="L155" s="14"/>
+      <c r="M155" s="14"/>
+      <c r="N155" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O155" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P155" s="14"/>
+      <c r="Q155" s="14"/>
+      <c r="R155" s="14"/>
+      <c r="S155" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 3); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" spans="1:19">
+      <c r="A156" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B156" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detailed</t>
+        </is>
+      </c>
+      <c r="C156" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Middleware health</t>
+        </is>
+      </c>
+      <c r="D156" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Middleware components on the selected server with their status</t>
+        </is>
+      </c>
+      <c r="E156" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="F156" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metrics</t>
+        </is>
+      </c>
+      <c r="G156" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metrics-system.process, metrics-windows.service, metricbeat</t>
+        </is>
+      </c>
+      <c r="H156" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Middleware Health (Table)</t>
+        </is>
+      </c>
+      <c r="I156" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Down = stopped or silent for 10 min. Health window control.</t>
+        </is>
+      </c>
+      <c r="J156" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">component, status, minutes since seen, server</t>
+        </is>
+      </c>
+      <c r="K156" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="L156" s="14"/>
+      <c r="M156" s="14"/>
+      <c r="N156" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O156" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P156" s="14"/>
+      <c r="Q156" s="14"/>
+      <c r="R156" s="14"/>
+      <c r="S156" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 3); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" spans="1:19">
+      <c r="A157" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B157" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detailed</t>
+        </is>
+      </c>
+      <c r="C157" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Database health</t>
+        </is>
+      </c>
+      <c r="D157" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Databases on the selected server with their status</t>
+        </is>
+      </c>
+      <c r="E157" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="F157" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metrics</t>
+        </is>
+      </c>
+      <c r="G157" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metricbeat (SQL Server), metrics-windows.service, metrics-system.process</t>
+        </is>
+      </c>
+      <c r="H157" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Database Health (Table)</t>
+        </is>
+      </c>
+      <c r="I157" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Down = stopped or silent for 10 min. Health window control.</t>
+        </is>
+      </c>
+      <c r="J157" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">database, status, minutes since seen, server</t>
+        </is>
+      </c>
+      <c r="K157" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="L157" s="14"/>
+      <c r="M157" s="14"/>
+      <c r="N157" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O157" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P157" s="14"/>
+      <c r="Q157" s="14"/>
+      <c r="R157" s="14"/>
+      <c r="S157" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 3); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" spans="1:19">
+      <c r="A158" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B158" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detailed</t>
+        </is>
+      </c>
+      <c r="C158" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server health</t>
+        </is>
+      </c>
+      <c r="D158" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reporting status, CPU 90th percentile, peak memory and fullest disk of the selected server</t>
+        </is>
+      </c>
+      <c r="E158" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">%</t>
+        </is>
+      </c>
+      <c r="F158" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metrics</t>
+        </is>
+      </c>
+      <c r="G158" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metrics-system.cpu, metrics-system.memory, metrics-system.filesystem</t>
+        </is>
+      </c>
+      <c r="H158" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server Health (Table)</t>
+        </is>
+      </c>
+      <c r="I158" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Amber from 80 %, red from 90 %. Health window control.</t>
+        </is>
+      </c>
+      <c r="J158" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">server, status, minutes since data, CPU p90, memory peak, disk max</t>
+        </is>
+      </c>
+      <c r="K158" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">%</t>
+        </is>
+      </c>
+      <c r="L158" s="14"/>
+      <c r="M158" s="14"/>
+      <c r="N158" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O158" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P158" s="14"/>
+      <c r="Q158" s="14"/>
+      <c r="R158" s="14"/>
+      <c r="S158" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 3); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" spans="1:19">
+      <c r="A159" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B159" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detailed</t>
+        </is>
+      </c>
+      <c r="C159" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">APM services on the server</t>
+        </is>
+      </c>
+      <c r="D159" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Production APM services that sent data from the selected server</t>
+        </is>
+      </c>
+      <c r="E159" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="F159" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">APM</t>
+        </is>
+      </c>
+      <c r="G159" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metrics-apm.internal</t>
+        </is>
+      </c>
+      <c r="H159" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">APM Services Health (Table)</t>
+        </is>
+      </c>
+      <c r="I159" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Health window control.</t>
+        </is>
+      </c>
+      <c r="J159" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">service, last data, environment</t>
+        </is>
+      </c>
+      <c r="K159" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="L159" s="14"/>
+      <c r="M159" s="14"/>
+      <c r="N159" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O159" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P159" s="14"/>
+      <c r="Q159" s="14"/>
+      <c r="R159" s="14"/>
+      <c r="S159" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 3); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" spans="1:19">
+      <c r="A160" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B160" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detailed</t>
+        </is>
+      </c>
+      <c r="C160" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Process health</t>
+        </is>
+      </c>
+      <c r="D160" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Windows services and middleware processes on the selected server, problems first</t>
+        </is>
+      </c>
+      <c r="E160" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="F160" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metrics</t>
+        </is>
+      </c>
+      <c r="G160" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metrics-windows.service, metrics-system.process</t>
+        </is>
+      </c>
+      <c r="H160" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Process Health (Table)</t>
+        </is>
+      </c>
+      <c r="I160" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stopped = an Automatic service not running; not seen = no report for 10 min.</t>
+        </is>
+      </c>
+      <c r="J160" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">process / service, status, kind, minutes since seen, owner</t>
+        </is>
+      </c>
+      <c r="K160" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="L160" s="14"/>
+      <c r="M160" s="14"/>
+      <c r="N160" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O160" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P160" s="14"/>
+      <c r="Q160" s="14"/>
+      <c r="R160" s="14"/>
+      <c r="S160" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 3); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" spans="1:19">
+      <c r="A161" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B161" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detailed</t>
+        </is>
+      </c>
+      <c r="C161" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Synthetics health</t>
+        </is>
+      </c>
+      <c r="D161" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Synthetic monitors that target the selected CI: latest status and down checks</t>
+        </is>
+      </c>
+      <c r="E161" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="F161" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">synthetics</t>
+        </is>
+      </c>
+      <c r="G161" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">synthetics-*</t>
+        </is>
+      </c>
+      <c r="H161" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Synthetics Health (Table)</t>
+        </is>
+      </c>
+      <c r="I161" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ping monitors enriched with the CI, or monitors on its host name.</t>
+        </is>
+      </c>
+      <c r="J161" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">monitor, type, status, down checks, location</t>
+        </is>
+      </c>
+      <c r="K161" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="L161" s="14"/>
+      <c r="M161" s="14"/>
+      <c r="N161" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O161" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P161" s="14"/>
+      <c r="Q161" s="14"/>
+      <c r="R161" s="14"/>
+      <c r="S161" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 3); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" spans="1:19">
+      <c r="A162" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM</t>
+        </is>
+      </c>
+      <c r="B162" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detailed</t>
+        </is>
+      </c>
+      <c r="C162" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Errors from the logs</t>
+        </is>
+      </c>
+      <c r="D162" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Warning-and-worse log lines from the selected CI, grouped by message</t>
+        </is>
+      </c>
+      <c r="E162" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">count</t>
+        </is>
+      </c>
+      <c r="F162" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">logs</t>
+        </is>
+      </c>
+      <c r="G162" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">logs-*syslog*, logs-jboss, logs-apm.error, logs-apm.app</t>
+        </is>
+      </c>
+      <c r="H162" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Errors from the Logs (Table)</t>
+        </is>
+      </c>
+      <c r="I162" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Numbers in messages replaced by #. Health window control.</t>
+        </is>
+      </c>
+      <c r="J162" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">count, severity, source, message, first / last seen</t>
+        </is>
+      </c>
+      <c r="K162" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">count</t>
+        </is>
+      </c>
+      <c r="L162" s="14"/>
+      <c r="M162" s="14"/>
+      <c r="N162" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="O162" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P162" s="14"/>
+      <c r="Q162" s="14"/>
+      <c r="R162" s="14"/>
+      <c r="S162" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIM V3 (30 Oct 2026): new KPI achieved in MIM V3 (section 3); not in the earlier MIM KPI list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" spans="1:19" customFormat="1" hidden="1">
+      <c r="A163" s="14" t="s">
+        <v>723</v>
+      </c>
+      <c r="B163" s="14" t="s">
+        <v>490</v>
+      </c>
+      <c r="C163" s="14" t="s">
+        <v>545</v>
+      </c>
+      <c r="D163" s="14" t="s">
+        <v>516</v>
+      </c>
+      <c r="E163" s="64" t="s">
+        <v>315</v>
+      </c>
+      <c r="F163" s="14" t="s">
+        <v>316</v>
+      </c>
+      <c r="G163" s="14" t="s">
+        <v>392</v>
+      </c>
+      <c r="H163" s="14" t="s">
+        <v>318</v>
+      </c>
+      <c r="I163" s="14" t="s">
+        <v>546</v>
+      </c>
+      <c r="J163" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="K163" s="14" t="s">
+        <v>315</v>
+      </c>
+      <c r="L163" s="14" t="e" vm="112">
+        <v>#VALUE!</v>
+      </c>
+      <c r="M163" s="14"/>
+      <c r="N163" s="14" t="s">
+        <v>408</v>
+      </c>
+      <c r="O163" s="14" t="s">
+        <v>301</v>
+      </c>
+      <c r="P163" s="14" t="s">
+        <v>547</v>
+      </c>
+      <c r="Q163" s="14"/>
+      <c r="R163" s="14"/>
+      <c r="S163" s="14"/>
+    </row>
+    <row r="164" spans="1:19" hidden="1">
+      <c r="A164" s="14" t="s">
+        <v>723</v>
+      </c>
+      <c r="B164" s="14" t="s">
+        <v>490</v>
+      </c>
+      <c r="C164" s="14" t="s">
+        <v>548</v>
+      </c>
+      <c r="D164" s="14" t="s">
+        <v>549</v>
+      </c>
+      <c r="E164" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="F164" s="14" t="s">
+        <v>297</v>
+      </c>
+      <c r="G164" s="14" t="s">
+        <v>298</v>
+      </c>
+      <c r="H164" s="14" t="s">
+        <v>304</v>
+      </c>
+      <c r="I164" s="14" t="s">
+        <v>550</v>
+      </c>
+      <c r="J164" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="K164" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="L164" s="14" t="e" vm="113">
+        <v>#VALUE!</v>
+      </c>
+      <c r="M164" s="14"/>
+      <c r="N164" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="O164" s="14" t="s">
+        <v>408</v>
+      </c>
+      <c r="P164" s="62" t="s">
+        <v>724</v>
+      </c>
+      <c r="Q164" s="14"/>
+      <c r="R164" s="14"/>
+      <c r="S164" s="14"/>
+    </row>
+    <row r="165" spans="1:19" hidden="1">
+      <c r="A165" s="14" t="s">
+        <v>723</v>
+      </c>
+      <c r="B165" s="14" t="s">
+        <v>490</v>
+      </c>
+      <c r="C165" s="14" t="s">
+        <v>551</v>
+      </c>
+      <c r="D165" s="14" t="s">
+        <v>552</v>
+      </c>
+      <c r="E165" s="14" t="s">
+        <v>553</v>
+      </c>
+      <c r="F165" s="14" t="s">
+        <v>297</v>
+      </c>
+      <c r="G165" s="14" t="s">
+        <v>554</v>
+      </c>
+      <c r="H165" s="14" t="s">
+        <v>318</v>
+      </c>
+      <c r="I165" s="14" t="s">
+        <v>555</v>
+      </c>
+      <c r="J165" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="K165" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="L165" s="14" t="e" vm="114">
+        <v>#VALUE!</v>
+      </c>
+      <c r="M165" s="14"/>
+      <c r="N165" s="14" t="s">
+        <v>408</v>
+      </c>
+      <c r="O165" s="14" t="s">
+        <v>408</v>
+      </c>
+      <c r="P165" s="62" t="s">
+        <v>725</v>
+      </c>
+      <c r="Q165" s="14"/>
+      <c r="R165" s="14"/>
+      <c r="S165" s="14"/>
+    </row>
+    <row r="166" spans="1:19" hidden="1">
+      <c r="A166" s="14" t="s">
+        <v>723</v>
+      </c>
+      <c r="B166" s="14" t="s">
+        <v>490</v>
+      </c>
+      <c r="C166" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="D166" s="14" t="s">
+        <v>726</v>
+      </c>
+      <c r="E166" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="F166" s="14" t="s">
+        <v>316</v>
+      </c>
+      <c r="G166" s="14" t="s">
+        <v>392</v>
+      </c>
+      <c r="H166" s="14" t="s">
+        <v>304</v>
+      </c>
+      <c r="I166" s="14" t="s">
+        <v>727</v>
+      </c>
+      <c r="J166" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="K166" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="L166" s="14" t="e" vm="115">
+        <v>#VALUE!</v>
+      </c>
+      <c r="M166" s="14"/>
+      <c r="N166" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="O166" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="P166" s="14"/>
+      <c r="Q166" s="14"/>
+      <c r="R166" s="14"/>
+      <c r="S166" s="14"/>
+    </row>
+    <row r="167" spans="1:19" hidden="1">
+      <c r="A167" s="14" t="s">
+        <v>723</v>
+      </c>
+      <c r="B167" s="14" t="s">
+        <v>490</v>
+      </c>
+      <c r="C167" s="14" t="s">
+        <v>557</v>
+      </c>
+      <c r="D167" s="14" t="s">
+        <v>558</v>
+      </c>
+      <c r="E167" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="F167" s="14" t="s">
+        <v>297</v>
+      </c>
+      <c r="G167" s="14" t="s">
+        <v>298</v>
+      </c>
+      <c r="H167" s="14" t="s">
+        <v>427</v>
+      </c>
+      <c r="I167" s="14" t="s">
+        <v>559</v>
+      </c>
+      <c r="J167" s="14" t="s">
+        <v>560</v>
+      </c>
+      <c r="K167" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="L167" s="14" t="e" vm="116">
+        <v>#VALUE!</v>
+      </c>
+      <c r="M167" s="14"/>
+      <c r="N167" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="O167" s="14" t="s">
+        <v>301</v>
+      </c>
+      <c r="P167" s="14" t="s">
+        <v>728</v>
+      </c>
+      <c r="Q167" s="14"/>
+      <c r="R167" s="14"/>
+      <c r="S167" s="14"/>
+    </row>
+    <row r="168" spans="1:19" hidden="1">
+      <c r="A168" s="14" t="s">
+        <v>723</v>
+      </c>
+      <c r="B168" s="14" t="s">
+        <v>490</v>
+      </c>
+      <c r="C168" s="14" t="s">
+        <v>729</v>
+      </c>
+      <c r="D168" s="14" t="s">
+        <v>562</v>
+      </c>
+      <c r="E168" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="F168" s="14" t="s">
+        <v>297</v>
+      </c>
+      <c r="G168" s="14" t="s">
+        <v>298</v>
+      </c>
+      <c r="H168" s="14" t="s">
+        <v>304</v>
+      </c>
+      <c r="I168" s="14" t="s">
+        <v>563</v>
+      </c>
+      <c r="J168" s="14" t="s">
+        <v>564</v>
+      </c>
+      <c r="K168" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="L168" s="14" t="e" vm="117">
+        <v>#VALUE!</v>
+      </c>
+      <c r="M168" s="14"/>
+      <c r="N168" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="O168" s="14" t="s">
+        <v>301</v>
+      </c>
+      <c r="P168" s="14" t="s">
+        <v>728</v>
+      </c>
+      <c r="Q168" s="14"/>
+      <c r="R168" s="14"/>
+      <c r="S168" s="14"/>
+    </row>
+    <row r="169" spans="1:19" hidden="1">
+      <c r="A169" s="14" t="s">
+        <v>723</v>
+      </c>
+      <c r="B169" s="14" t="s">
+        <v>490</v>
+      </c>
+      <c r="C169" s="14" t="s">
+        <v>566</v>
+      </c>
+      <c r="D169" s="14" t="s">
+        <v>567</v>
+      </c>
+      <c r="E169" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="F169" s="14" t="s">
+        <v>297</v>
+      </c>
+      <c r="G169" s="14" t="s">
+        <v>426</v>
+      </c>
+      <c r="H169" s="14" t="s">
+        <v>359</v>
+      </c>
+      <c r="I169" s="14" t="s">
+        <v>568</v>
+      </c>
+      <c r="J169" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="K169" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="L169" s="14" t="e" vm="118">
+        <v>#VALUE!</v>
+      </c>
+      <c r="M169" s="14"/>
+      <c r="N169" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="O169" s="14" t="s">
+        <v>408</v>
+      </c>
+      <c r="P169" s="14" t="s">
+        <v>569</v>
+      </c>
+      <c r="Q169" s="14"/>
+      <c r="R169" s="14"/>
+      <c r="S169" s="14"/>
+    </row>
+    <row r="170" spans="1:19" hidden="1">
+      <c r="A170" s="14" t="s">
+        <v>723</v>
+      </c>
+      <c r="B170" s="14" t="s">
+        <v>490</v>
+      </c>
+      <c r="C170" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="D170" s="14" t="s">
+        <v>570</v>
+      </c>
+      <c r="E170" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="F170" s="14" t="s">
+        <v>316</v>
+      </c>
+      <c r="G170" s="14" t="s">
+        <v>316</v>
+      </c>
+      <c r="H170" s="14" t="s">
+        <v>427</v>
+      </c>
+      <c r="I170" s="14" t="s">
+        <v>571</v>
+      </c>
+      <c r="J170" s="14"/>
+      <c r="K170" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="L170" s="14" t="e" vm="119">
+        <v>#VALUE!</v>
+      </c>
+      <c r="M170" s="14"/>
+      <c r="N170" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="O170" s="14" t="s">
+        <v>408</v>
+      </c>
+      <c r="P170" s="14" t="s">
+        <v>572</v>
+      </c>
+      <c r="Q170" s="14"/>
+      <c r="R170" s="14"/>
+      <c r="S170" s="14"/>
+    </row>
+    <row r="171" spans="1:19" hidden="1">
+      <c r="A171" s="14" t="s">
+        <v>723</v>
+      </c>
+      <c r="B171" s="14" t="s">
+        <v>490</v>
+      </c>
+      <c r="C171" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="D171" s="59" t="s">
+        <v>573</v>
+      </c>
+      <c r="E171" s="14" t="s">
+        <v>315</v>
+      </c>
+      <c r="F171" s="14" t="s">
+        <v>334</v>
+      </c>
+      <c r="G171" s="14" t="s">
+        <v>574</v>
+      </c>
+      <c r="H171" s="14" t="s">
+        <v>304</v>
+      </c>
+      <c r="I171" s="14" t="s">
+        <v>575</v>
+      </c>
+      <c r="J171" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="K171" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="L171" s="14" t="e" vm="120">
+        <v>#VALUE!</v>
+      </c>
+      <c r="M171" s="14"/>
+      <c r="N171" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="O171" s="14" t="s">
+        <v>408</v>
+      </c>
+      <c r="P171" s="14" t="s">
+        <v>730</v>
+      </c>
+      <c r="Q171" s="14"/>
+      <c r="R171" s="14"/>
+      <c r="S171" s="14"/>
+    </row>
+    <row r="172" spans="1:19" hidden="1">
+      <c r="A172" s="14" t="s">
+        <v>723</v>
+      </c>
+      <c r="B172" s="14" t="s">
+        <v>490</v>
+      </c>
+      <c r="C172" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="D172" s="14" t="s">
+        <v>577</v>
+      </c>
+      <c r="E172" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="F172" s="14" t="s">
+        <v>297</v>
+      </c>
+      <c r="G172" s="59" t="s">
+        <v>298</v>
+      </c>
+      <c r="H172" s="14" t="s">
+        <v>427</v>
+      </c>
+      <c r="I172" s="14" t="s">
+        <v>578</v>
+      </c>
+      <c r="J172" s="14" t="s">
+        <v>564</v>
+      </c>
+      <c r="K172" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="L172" s="14" t="e" vm="121">
+        <v>#VALUE!</v>
+      </c>
+      <c r="M172" s="14"/>
+      <c r="N172" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="O172" s="14" t="s">
+        <v>408</v>
+      </c>
+      <c r="P172" s="65" t="s">
+        <v>731</v>
+      </c>
+      <c r="Q172" s="14"/>
+      <c r="R172" s="14"/>
+      <c r="S172" s="14"/>
+    </row>
+    <row r="173" spans="1:19" hidden="1">
+      <c r="A173" s="14" t="s">
+        <v>723</v>
+      </c>
+      <c r="B173" s="14" t="s">
+        <v>490</v>
+      </c>
+      <c r="C173" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="D173" s="14" t="s">
+        <v>580</v>
+      </c>
+      <c r="E173" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="F173" s="14" t="s">
+        <v>297</v>
+      </c>
+      <c r="G173" s="59" t="s">
+        <v>298</v>
+      </c>
+      <c r="H173" s="14" t="s">
+        <v>304</v>
+      </c>
+      <c r="I173" s="14" t="s">
+        <v>581</v>
+      </c>
+      <c r="J173" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="K173" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="L173" s="14" t="e" vm="122">
+        <v>#VALUE!</v>
+      </c>
+      <c r="M173" s="14"/>
+      <c r="N173" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="O173" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="P173" s="61" t="s">
+        <v>582</v>
+      </c>
+      <c r="Q173" s="14"/>
+      <c r="R173" s="14"/>
+      <c r="S173" s="14"/>
+    </row>
+    <row r="174" spans="1:19" hidden="1">
+      <c r="A174" s="14" t="s">
+        <v>723</v>
+      </c>
+      <c r="B174" s="14" t="s">
+        <v>490</v>
+      </c>
+      <c r="C174" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="D174" s="14" t="s">
+        <v>583</v>
+      </c>
+      <c r="E174" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="F174" s="14" t="s">
+        <v>297</v>
+      </c>
+      <c r="G174" s="59" t="s">
+        <v>298</v>
+      </c>
+      <c r="H174" s="14" t="s">
+        <v>318</v>
+      </c>
+      <c r="I174" s="14" t="s">
+        <v>555</v>
+      </c>
+      <c r="J174" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="K174" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="L174" s="14" t="e" vm="123">
+        <v>#VALUE!</v>
+      </c>
+      <c r="M174" s="14"/>
+      <c r="N174" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="O174" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="P174" s="61" t="s">
+        <v>582</v>
+      </c>
+      <c r="Q174" s="14"/>
+      <c r="R174" s="14"/>
+      <c r="S174" s="14"/>
+    </row>
+    <row r="175" spans="1:19" hidden="1">
+      <c r="A175" s="6" t="s">
         <v>292</v>
       </c>
-      <c r="B152" s="6" t="s">
+      <c r="B175" s="6" t="s">
         <v>490</v>
       </c>
-      <c r="C152" s="6" t="s">
+      <c r="C175" s="6" t="s">
         <v>732</v>
       </c>
-      <c r="D152" s="69" t="s">
+      <c r="D175" s="69" t="s">
         <v>732</v>
       </c>
-      <c r="E152" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="F152" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="G152" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="H152" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="I152" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="J152" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="K152" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="L152" s="6" t="e" vm="124">
+      <c r="E175" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="F175" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="G175" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="H175" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="I175" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="J175" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="K175" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="L175" s="6" t="e" vm="124">
         <v>#VALUE!</v>
       </c>
-      <c r="M152" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="N152" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="O152" s="6" t="s">
+      <c r="M175" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="N175" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="O175" s="6" t="s">
         <v>301</v>
       </c>
-      <c r="P152" s="6" t="s">
+      <c r="P175" s="6" t="s">
         <v>733</v>
       </c>
-      <c r="Q152" s="10">
+      <c r="Q175" s="10">
         <v>46307</v>
       </c>
-      <c r="R152" s="6" t="s">
+      <c r="R175" s="6" t="s">
         <v>301</v>
       </c>
-      <c r="S152" s="6"/>
+      <c r="S175" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S152" xr:uid="{5F8E8311-F168-4ED2-854F-F6B1C5578AEA}">
+  <autoFilter ref="A1:S175" xr:uid="{5F8E8311-F168-4ED2-854F-F6B1C5578AEA}">
     <filterColumn colId="0">
       <filters>
         <filter val="MIM"/>
@@ -20226,27 +22109,27 @@
       <formula>NOT(ISERROR(SEARCH("Fail",N2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N113:O143">
+  <conditionalFormatting sqref="N113:O166">
     <cfRule type="containsText" dxfId="4" priority="17" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",N113)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N146:O149">
+  <conditionalFormatting sqref="N169:O172">
     <cfRule type="containsText" dxfId="3" priority="19" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",N146)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Fail",N169)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O106:O112 N144:N146">
+  <conditionalFormatting sqref="O106:O112 N167:N169">
     <cfRule type="containsText" dxfId="2" priority="29" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",N106)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O144:O145">
+  <conditionalFormatting sqref="O167:O168">
     <cfRule type="containsText" dxfId="1" priority="21" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",O144)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Fail",O167)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R3 R5:R75 R77:R149 N150:N151 N152:O152">
+  <conditionalFormatting sqref="R3 R5:R75 R77:R172 N173:N174 N175:O175">
     <cfRule type="containsText" dxfId="0" priority="20" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",N3)))</formula>
     </cfRule>

</xml_diff>